<commit_message>
fix: monto de operaciones inter compañía y duplicación de razón social
- excelOperationsParser: la Tabla 3 (Transacciones Inter compañía) sumaba
  filas de la sección de Egreso y renglones sin código de operación junto
  con la de Ingreso, inflando el monto en pesos. Ahora solo se suman filas
  de la sección de Ingreso que tengan el código ("Cod") diligenciado.
- exactTemplateMapper/masterTemplate: evita que el barrido final de
  variantes de "END GAME" duplique la razón social cuando el contribuyente
  real coincide con el nombre de la plantilla base.
</commit_message>
<xml_diff>
--- a/Cpanel/public_html/demo-precios-transferencia/Archivos Prueba/Información Operaciones PT 2025-2 modificado cr.xlsx
+++ b/Cpanel/public_html/demo-precios-transferencia/Archivos Prueba/Información Operaciones PT 2025-2 modificado cr.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\.shortcut-targets-by-id\1AhE4eqM8c6mfTdaitS_hpQkb28vUXOO8\4. PRECIOS TRANSFERENCIA\AÑO 2025\End Game\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Precios de Transferencia\Cpanel\public_html\demo-precios-transferencia\Archivos Prueba\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A95A0667-56C6-437D-B01F-137B6C2A6787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{204A5DF6-9F72-4BEA-B46E-4A9E1344C960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,23 @@
     <definedName name="IQ_YTD">3000</definedName>
     <definedName name="IQ_YTDMONTH" hidden="1">130000</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="9.9999999999994451E-4"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -721,7 +737,7 @@
     <numFmt numFmtId="173" formatCode="0.000%\ &quot;Efectivo Anual&quot;"/>
     <numFmt numFmtId="174" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="43">
+  <fonts count="44">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -983,6 +999,12 @@
       <b/>
       <sz val="13"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1712,7 +1734,7 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="25" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="39" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="163">
+  <cellXfs count="164">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2008,13 +2030,53 @@
     <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="38" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="16" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2051,52 +2113,12 @@
     <xf numFmtId="0" fontId="11" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="37" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2112,6 +2134,7 @@
     <xf numFmtId="3" fontId="32" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="222">
     <cellStyle name="0,0_x000d__x000a_NA_x000d__x000a_" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -2920,38 +2943,38 @@
       <c r="M1" s="3"/>
     </row>
     <row r="2" spans="1:13" s="27" customFormat="1" ht="18">
-      <c r="A2" s="130" t="s">
+      <c r="A2" s="144" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
-      <c r="H2" s="130"/>
-      <c r="I2" s="130"/>
-      <c r="J2" s="130"/>
-      <c r="K2" s="130"/>
-      <c r="L2" s="130"/>
-      <c r="M2" s="130"/>
+      <c r="B2" s="144"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="144"/>
+      <c r="J2" s="144"/>
+      <c r="K2" s="144"/>
+      <c r="L2" s="144"/>
+      <c r="M2" s="144"/>
     </row>
     <row r="3" spans="1:13" s="27" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A3" s="130" t="s">
+      <c r="A3" s="144" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="130"/>
-      <c r="C3" s="130"/>
-      <c r="D3" s="130"/>
-      <c r="E3" s="130"/>
-      <c r="F3" s="130"/>
-      <c r="G3" s="130"/>
-      <c r="H3" s="130"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="130"/>
-      <c r="K3" s="130"/>
-      <c r="L3" s="130"/>
-      <c r="M3" s="130"/>
+      <c r="B3" s="144"/>
+      <c r="C3" s="144"/>
+      <c r="D3" s="144"/>
+      <c r="E3" s="144"/>
+      <c r="F3" s="144"/>
+      <c r="G3" s="144"/>
+      <c r="H3" s="144"/>
+      <c r="I3" s="144"/>
+      <c r="J3" s="144"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="144"/>
+      <c r="M3" s="144"/>
     </row>
     <row r="4" spans="1:13" s="27" customFormat="1" ht="15" customHeight="1">
       <c r="A4" s="1"/>
@@ -2988,16 +3011,16 @@
       <c r="B6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="141"/>
-      <c r="D6" s="141"/>
-      <c r="E6" s="141"/>
-      <c r="F6" s="141"/>
-      <c r="G6" s="141"/>
-      <c r="H6" s="141"/>
-      <c r="I6" s="141"/>
-      <c r="J6" s="141"/>
-      <c r="K6" s="141"/>
-      <c r="L6" s="141"/>
+      <c r="C6" s="155"/>
+      <c r="D6" s="155"/>
+      <c r="E6" s="155"/>
+      <c r="F6" s="155"/>
+      <c r="G6" s="155"/>
+      <c r="H6" s="155"/>
+      <c r="I6" s="155"/>
+      <c r="J6" s="155"/>
+      <c r="K6" s="155"/>
+      <c r="L6" s="155"/>
       <c r="M6" s="3"/>
     </row>
     <row r="7" spans="1:13" s="27" customFormat="1" ht="15.75">
@@ -3007,7 +3030,7 @@
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="1"/>
+      <c r="G7" s="163"/>
       <c r="H7" s="1"/>
       <c r="I7" s="10"/>
       <c r="J7" s="1"/>
@@ -3028,10 +3051,10 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
-      <c r="I8" s="150" t="s">
+      <c r="I8" s="156" t="s">
         <v>36</v>
       </c>
-      <c r="J8" s="150"/>
+      <c r="J8" s="156"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="3"/>
@@ -3053,50 +3076,50 @@
     </row>
     <row r="10" spans="1:13" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A10" s="35"/>
-      <c r="B10" s="142" t="s">
+      <c r="B10" s="131" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="142" t="s">
+      <c r="C10" s="131" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="142" t="s">
+      <c r="D10" s="131" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="127" t="s">
+      <c r="E10" s="129" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="142" t="s">
+      <c r="F10" s="131" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="142" t="s">
+      <c r="G10" s="131" t="s">
         <v>24</v>
       </c>
       <c r="H10" s="1"/>
-      <c r="I10" s="152" t="s">
+      <c r="I10" s="136" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="142" t="s">
+      <c r="J10" s="131" t="s">
         <v>32</v>
       </c>
       <c r="K10" s="120"/>
-      <c r="L10" s="142" t="s">
+      <c r="L10" s="131" t="s">
         <v>37</v>
       </c>
       <c r="M10" s="3"/>
     </row>
     <row r="11" spans="1:13" s="27" customFormat="1" ht="28.35" customHeight="1">
       <c r="A11" s="35"/>
-      <c r="B11" s="143"/>
-      <c r="C11" s="143"/>
-      <c r="D11" s="143"/>
-      <c r="E11" s="155"/>
-      <c r="F11" s="143"/>
-      <c r="G11" s="143"/>
+      <c r="B11" s="132"/>
+      <c r="C11" s="132"/>
+      <c r="D11" s="132"/>
+      <c r="E11" s="130"/>
+      <c r="F11" s="132"/>
+      <c r="G11" s="132"/>
       <c r="H11" s="1"/>
-      <c r="I11" s="153"/>
-      <c r="J11" s="143"/>
+      <c r="I11" s="137"/>
+      <c r="J11" s="132"/>
       <c r="K11" s="120"/>
-      <c r="L11" s="143"/>
+      <c r="L11" s="132"/>
       <c r="M11" s="3"/>
     </row>
     <row r="12" spans="1:13" s="27" customFormat="1" ht="15.95" customHeight="1">
@@ -3116,7 +3139,9 @@
       <c r="F12" s="109" t="s">
         <v>175</v>
       </c>
-      <c r="G12" s="109"/>
+      <c r="G12" s="109">
+        <v>7</v>
+      </c>
       <c r="H12" s="108"/>
       <c r="I12" s="112">
         <v>1007</v>
@@ -3260,10 +3285,10 @@
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
-      <c r="I20" s="150" t="s">
+      <c r="I20" s="156" t="s">
         <v>36</v>
       </c>
-      <c r="J20" s="150"/>
+      <c r="J20" s="156"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
       <c r="M20" s="3"/>
@@ -3285,53 +3310,53 @@
     </row>
     <row r="22" spans="1:13" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A22" s="35"/>
-      <c r="B22" s="142" t="s">
+      <c r="B22" s="131" t="s">
         <v>28</v>
       </c>
-      <c r="C22" s="142" t="s">
+      <c r="C22" s="131" t="s">
         <v>26</v>
       </c>
-      <c r="D22" s="142" t="s">
+      <c r="D22" s="131" t="s">
         <v>25</v>
       </c>
-      <c r="E22" s="127" t="s">
+      <c r="E22" s="129" t="s">
         <v>114</v>
       </c>
-      <c r="F22" s="142" t="s">
+      <c r="F22" s="131" t="s">
         <v>27</v>
       </c>
-      <c r="G22" s="142" t="s">
+      <c r="G22" s="131" t="s">
         <v>24</v>
       </c>
       <c r="H22" s="1"/>
-      <c r="I22" s="152" t="s">
+      <c r="I22" s="136" t="s">
         <v>31</v>
       </c>
-      <c r="J22" s="142" t="s">
+      <c r="J22" s="131" t="s">
         <v>32</v>
       </c>
       <c r="K22" s="120"/>
-      <c r="L22" s="142" t="s">
+      <c r="L22" s="131" t="s">
         <v>38</v>
       </c>
-      <c r="M22" s="142" t="s">
+      <c r="M22" s="131" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:13" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A23" s="35"/>
-      <c r="B23" s="143"/>
-      <c r="C23" s="143"/>
-      <c r="D23" s="143"/>
-      <c r="E23" s="155"/>
-      <c r="F23" s="143"/>
-      <c r="G23" s="143"/>
+      <c r="B23" s="132"/>
+      <c r="C23" s="132"/>
+      <c r="D23" s="132"/>
+      <c r="E23" s="130"/>
+      <c r="F23" s="132"/>
+      <c r="G23" s="132"/>
       <c r="H23" s="1"/>
-      <c r="I23" s="153"/>
-      <c r="J23" s="143"/>
+      <c r="I23" s="137"/>
+      <c r="J23" s="132"/>
       <c r="K23" s="120"/>
-      <c r="L23" s="143"/>
-      <c r="M23" s="143"/>
+      <c r="L23" s="132"/>
+      <c r="M23" s="132"/>
     </row>
     <row r="24" spans="1:13" s="27" customFormat="1" ht="15.75">
       <c r="A24" s="35"/>
@@ -3495,10 +3520,10 @@
       <c r="A33" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="B33" s="131" t="s">
+      <c r="B33" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C33" s="131"/>
+      <c r="C33" s="145"/>
       <c r="D33" s="1"/>
       <c r="E33" s="1"/>
       <c r="F33" s="29"/>
@@ -3527,53 +3552,53 @@
     </row>
     <row r="35" spans="1:13" s="27" customFormat="1" ht="15.75">
       <c r="A35" s="35"/>
-      <c r="B35" s="142" t="s">
+      <c r="B35" s="131" t="s">
         <v>28</v>
       </c>
-      <c r="C35" s="142" t="s">
+      <c r="C35" s="131" t="s">
         <v>26</v>
       </c>
-      <c r="D35" s="142" t="s">
+      <c r="D35" s="131" t="s">
         <v>113</v>
       </c>
-      <c r="E35" s="127" t="s">
+      <c r="E35" s="129" t="s">
         <v>114</v>
       </c>
-      <c r="F35" s="142" t="s">
+      <c r="F35" s="131" t="s">
         <v>27</v>
       </c>
-      <c r="G35" s="142" t="s">
+      <c r="G35" s="131" t="s">
         <v>24</v>
       </c>
-      <c r="H35" s="144" t="s">
+      <c r="H35" s="138" t="s">
         <v>138</v>
       </c>
-      <c r="I35" s="145"/>
-      <c r="J35" s="144" t="s">
+      <c r="I35" s="139"/>
+      <c r="J35" s="138" t="s">
         <v>139</v>
       </c>
-      <c r="K35" s="145"/>
-      <c r="L35" s="127" t="s">
+      <c r="K35" s="139"/>
+      <c r="L35" s="129" t="s">
         <v>140</v>
       </c>
-      <c r="M35" s="127" t="s">
+      <c r="M35" s="129" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="36" spans="1:13" s="27" customFormat="1" ht="15.75">
       <c r="A36" s="35"/>
-      <c r="B36" s="143"/>
-      <c r="C36" s="143"/>
-      <c r="D36" s="143"/>
-      <c r="E36" s="155"/>
-      <c r="F36" s="143"/>
-      <c r="G36" s="143"/>
-      <c r="H36" s="146"/>
-      <c r="I36" s="147"/>
-      <c r="J36" s="146"/>
-      <c r="K36" s="147"/>
-      <c r="L36" s="128"/>
-      <c r="M36" s="128"/>
+      <c r="B36" s="132"/>
+      <c r="C36" s="132"/>
+      <c r="D36" s="132"/>
+      <c r="E36" s="130"/>
+      <c r="F36" s="132"/>
+      <c r="G36" s="132"/>
+      <c r="H36" s="140"/>
+      <c r="I36" s="141"/>
+      <c r="J36" s="140"/>
+      <c r="K36" s="141"/>
+      <c r="L36" s="135"/>
+      <c r="M36" s="135"/>
     </row>
     <row r="37" spans="1:13" s="27" customFormat="1" ht="15.75">
       <c r="A37" s="35"/>
@@ -3583,10 +3608,10 @@
       <c r="E37" s="6"/>
       <c r="F37" s="6"/>
       <c r="G37" s="6"/>
-      <c r="H37" s="129"/>
-      <c r="I37" s="129"/>
-      <c r="J37" s="129"/>
-      <c r="K37" s="129"/>
+      <c r="H37" s="134"/>
+      <c r="I37" s="134"/>
+      <c r="J37" s="134"/>
+      <c r="K37" s="134"/>
       <c r="L37" s="7"/>
       <c r="M37" s="7"/>
     </row>
@@ -3598,10 +3623,10 @@
       <c r="E38" s="6"/>
       <c r="F38" s="6"/>
       <c r="G38" s="6"/>
-      <c r="H38" s="129"/>
-      <c r="I38" s="129"/>
-      <c r="J38" s="129"/>
-      <c r="K38" s="129"/>
+      <c r="H38" s="134"/>
+      <c r="I38" s="134"/>
+      <c r="J38" s="134"/>
+      <c r="K38" s="134"/>
       <c r="L38" s="7"/>
       <c r="M38" s="7"/>
     </row>
@@ -3613,10 +3638,10 @@
       <c r="E39" s="6"/>
       <c r="F39" s="6"/>
       <c r="G39" s="6"/>
-      <c r="H39" s="129"/>
-      <c r="I39" s="129"/>
-      <c r="J39" s="129"/>
-      <c r="K39" s="129"/>
+      <c r="H39" s="134"/>
+      <c r="I39" s="134"/>
+      <c r="J39" s="134"/>
+      <c r="K39" s="134"/>
       <c r="L39" s="7"/>
       <c r="M39" s="7"/>
     </row>
@@ -3628,10 +3653,10 @@
       <c r="E40" s="6"/>
       <c r="F40" s="6"/>
       <c r="G40" s="36"/>
-      <c r="H40" s="129"/>
-      <c r="I40" s="129"/>
-      <c r="J40" s="154"/>
-      <c r="K40" s="154"/>
+      <c r="H40" s="134"/>
+      <c r="I40" s="134"/>
+      <c r="J40" s="143"/>
+      <c r="K40" s="143"/>
       <c r="L40" s="7"/>
       <c r="M40" s="7"/>
     </row>
@@ -3643,10 +3668,10 @@
       <c r="E41" s="6"/>
       <c r="F41" s="6"/>
       <c r="G41" s="6"/>
-      <c r="H41" s="129"/>
-      <c r="I41" s="129"/>
-      <c r="J41" s="129"/>
-      <c r="K41" s="129"/>
+      <c r="H41" s="134"/>
+      <c r="I41" s="134"/>
+      <c r="J41" s="134"/>
+      <c r="K41" s="134"/>
       <c r="L41" s="7"/>
       <c r="M41" s="7"/>
     </row>
@@ -3658,10 +3683,10 @@
       <c r="E42" s="6"/>
       <c r="F42" s="6"/>
       <c r="G42" s="6"/>
-      <c r="H42" s="129"/>
-      <c r="I42" s="129"/>
-      <c r="J42" s="129"/>
-      <c r="K42" s="129"/>
+      <c r="H42" s="134"/>
+      <c r="I42" s="134"/>
+      <c r="J42" s="134"/>
+      <c r="K42" s="134"/>
       <c r="L42" s="7"/>
       <c r="M42" s="7"/>
     </row>
@@ -3716,20 +3741,20 @@
     </row>
     <row r="46" spans="1:13" s="27" customFormat="1" ht="39.75" customHeight="1">
       <c r="A46" s="1"/>
-      <c r="B46" s="151" t="s">
+      <c r="B46" s="157" t="s">
         <v>142</v>
       </c>
-      <c r="C46" s="151"/>
-      <c r="D46" s="151"/>
-      <c r="E46" s="151"/>
-      <c r="F46" s="151"/>
-      <c r="G46" s="151"/>
-      <c r="H46" s="151"/>
-      <c r="I46" s="151"/>
-      <c r="J46" s="151"/>
-      <c r="K46" s="151"/>
-      <c r="L46" s="151"/>
-      <c r="M46" s="151"/>
+      <c r="C46" s="157"/>
+      <c r="D46" s="157"/>
+      <c r="E46" s="157"/>
+      <c r="F46" s="157"/>
+      <c r="G46" s="157"/>
+      <c r="H46" s="157"/>
+      <c r="I46" s="157"/>
+      <c r="J46" s="157"/>
+      <c r="K46" s="157"/>
+      <c r="L46" s="157"/>
+      <c r="M46" s="157"/>
     </row>
     <row r="47" spans="1:13" s="27" customFormat="1" ht="16.5" customHeight="1">
       <c r="A47" s="1"/>
@@ -3748,53 +3773,53 @@
     </row>
     <row r="48" spans="1:13" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A48" s="1"/>
-      <c r="B48" s="148" t="s">
+      <c r="B48" s="127" t="s">
         <v>28</v>
       </c>
-      <c r="C48" s="148" t="s">
+      <c r="C48" s="127" t="s">
         <v>26</v>
       </c>
-      <c r="D48" s="148" t="s">
+      <c r="D48" s="127" t="s">
         <v>25</v>
       </c>
-      <c r="E48" s="127" t="s">
+      <c r="E48" s="129" t="s">
         <v>114</v>
       </c>
-      <c r="F48" s="148" t="s">
+      <c r="F48" s="127" t="s">
         <v>27</v>
       </c>
-      <c r="G48" s="148" t="s">
+      <c r="G48" s="127" t="s">
         <v>24</v>
       </c>
-      <c r="H48" s="144" t="s">
+      <c r="H48" s="138" t="s">
         <v>138</v>
       </c>
-      <c r="I48" s="145"/>
-      <c r="J48" s="144" t="s">
+      <c r="I48" s="139"/>
+      <c r="J48" s="138" t="s">
         <v>139</v>
       </c>
-      <c r="K48" s="145"/>
-      <c r="L48" s="127" t="s">
+      <c r="K48" s="139"/>
+      <c r="L48" s="129" t="s">
         <v>140</v>
       </c>
-      <c r="M48" s="127" t="s">
+      <c r="M48" s="129" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="49" spans="1:257" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A49" s="1"/>
-      <c r="B49" s="149"/>
-      <c r="C49" s="149"/>
-      <c r="D49" s="149"/>
-      <c r="E49" s="155"/>
-      <c r="F49" s="149"/>
-      <c r="G49" s="149"/>
-      <c r="H49" s="146"/>
-      <c r="I49" s="147"/>
-      <c r="J49" s="146"/>
-      <c r="K49" s="147"/>
-      <c r="L49" s="128"/>
-      <c r="M49" s="128"/>
+      <c r="B49" s="128"/>
+      <c r="C49" s="128"/>
+      <c r="D49" s="128"/>
+      <c r="E49" s="130"/>
+      <c r="F49" s="128"/>
+      <c r="G49" s="128"/>
+      <c r="H49" s="140"/>
+      <c r="I49" s="141"/>
+      <c r="J49" s="140"/>
+      <c r="K49" s="141"/>
+      <c r="L49" s="135"/>
+      <c r="M49" s="135"/>
     </row>
     <row r="50" spans="1:257" s="108" customFormat="1" ht="15.95" customHeight="1">
       <c r="B50" s="70"/>
@@ -3802,10 +3827,10 @@
       <c r="D50" s="109"/>
       <c r="F50" s="114"/>
       <c r="G50" s="110"/>
-      <c r="H50" s="156"/>
-      <c r="I50" s="156"/>
-      <c r="J50" s="156"/>
-      <c r="K50" s="156"/>
+      <c r="H50" s="142"/>
+      <c r="I50" s="142"/>
+      <c r="J50" s="142"/>
+      <c r="K50" s="142"/>
       <c r="L50" s="109"/>
       <c r="M50" s="109"/>
     </row>
@@ -3817,10 +3842,10 @@
       <c r="E51" s="6"/>
       <c r="F51" s="6"/>
       <c r="G51" s="6"/>
-      <c r="H51" s="129"/>
-      <c r="I51" s="129"/>
-      <c r="J51" s="129"/>
-      <c r="K51" s="129"/>
+      <c r="H51" s="134"/>
+      <c r="I51" s="134"/>
+      <c r="J51" s="134"/>
+      <c r="K51" s="134"/>
       <c r="L51" s="7"/>
       <c r="M51" s="7"/>
     </row>
@@ -3832,10 +3857,10 @@
       <c r="E52" s="6"/>
       <c r="F52" s="6"/>
       <c r="G52" s="6"/>
-      <c r="H52" s="129"/>
-      <c r="I52" s="129"/>
-      <c r="J52" s="129"/>
-      <c r="K52" s="129"/>
+      <c r="H52" s="134"/>
+      <c r="I52" s="134"/>
+      <c r="J52" s="134"/>
+      <c r="K52" s="134"/>
       <c r="L52" s="7"/>
       <c r="M52" s="7"/>
     </row>
@@ -3847,10 +3872,10 @@
       <c r="E53" s="6"/>
       <c r="F53" s="6"/>
       <c r="G53" s="6"/>
-      <c r="H53" s="129"/>
-      <c r="I53" s="129"/>
-      <c r="J53" s="129"/>
-      <c r="K53" s="129"/>
+      <c r="H53" s="134"/>
+      <c r="I53" s="134"/>
+      <c r="J53" s="134"/>
+      <c r="K53" s="134"/>
       <c r="L53" s="7"/>
       <c r="M53" s="7"/>
     </row>
@@ -3862,10 +3887,10 @@
       <c r="E54" s="6"/>
       <c r="F54" s="6"/>
       <c r="G54" s="6"/>
-      <c r="H54" s="129"/>
-      <c r="I54" s="129"/>
-      <c r="J54" s="129"/>
-      <c r="K54" s="129"/>
+      <c r="H54" s="134"/>
+      <c r="I54" s="134"/>
+      <c r="J54" s="134"/>
+      <c r="K54" s="134"/>
       <c r="L54" s="7"/>
       <c r="M54" s="7"/>
     </row>
@@ -3877,10 +3902,10 @@
       <c r="E55" s="6"/>
       <c r="F55" s="6"/>
       <c r="G55" s="6"/>
-      <c r="H55" s="129"/>
-      <c r="I55" s="129"/>
-      <c r="J55" s="129"/>
-      <c r="K55" s="129"/>
+      <c r="H55" s="134"/>
+      <c r="I55" s="134"/>
+      <c r="J55" s="134"/>
+      <c r="K55" s="134"/>
       <c r="L55" s="7"/>
       <c r="M55" s="7"/>
     </row>
@@ -3900,21 +3925,21 @@
       <c r="M56" s="3"/>
     </row>
     <row r="57" spans="1:257" s="1" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A57" s="132" t="s">
+      <c r="A57" s="146" t="s">
         <v>21</v>
       </c>
-      <c r="B57" s="133"/>
-      <c r="C57" s="133"/>
-      <c r="D57" s="133"/>
-      <c r="E57" s="133"/>
-      <c r="F57" s="133"/>
-      <c r="G57" s="133"/>
-      <c r="H57" s="133"/>
-      <c r="I57" s="133"/>
-      <c r="J57" s="133"/>
-      <c r="K57" s="133"/>
-      <c r="L57" s="133"/>
-      <c r="M57" s="134"/>
+      <c r="B57" s="147"/>
+      <c r="C57" s="147"/>
+      <c r="D57" s="147"/>
+      <c r="E57" s="147"/>
+      <c r="F57" s="147"/>
+      <c r="G57" s="147"/>
+      <c r="H57" s="147"/>
+      <c r="I57" s="147"/>
+      <c r="J57" s="147"/>
+      <c r="K57" s="147"/>
+      <c r="L57" s="147"/>
+      <c r="M57" s="148"/>
       <c r="N57" s="27"/>
       <c r="O57" s="27"/>
       <c r="P57" s="27"/>
@@ -4161,49 +4186,49 @@
       <c r="IW57" s="27"/>
     </row>
     <row r="58" spans="1:257" s="27" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A58" s="135"/>
-      <c r="B58" s="136"/>
-      <c r="C58" s="136"/>
-      <c r="D58" s="136"/>
-      <c r="E58" s="136"/>
-      <c r="F58" s="136"/>
-      <c r="G58" s="136"/>
-      <c r="H58" s="136"/>
-      <c r="I58" s="136"/>
-      <c r="J58" s="136"/>
-      <c r="K58" s="136"/>
-      <c r="L58" s="136"/>
-      <c r="M58" s="137"/>
+      <c r="A58" s="149"/>
+      <c r="B58" s="150"/>
+      <c r="C58" s="150"/>
+      <c r="D58" s="150"/>
+      <c r="E58" s="150"/>
+      <c r="F58" s="150"/>
+      <c r="G58" s="150"/>
+      <c r="H58" s="150"/>
+      <c r="I58" s="150"/>
+      <c r="J58" s="150"/>
+      <c r="K58" s="150"/>
+      <c r="L58" s="150"/>
+      <c r="M58" s="151"/>
     </row>
     <row r="59" spans="1:257" s="27" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A59" s="135"/>
-      <c r="B59" s="136"/>
-      <c r="C59" s="136"/>
-      <c r="D59" s="136"/>
-      <c r="E59" s="136"/>
-      <c r="F59" s="136"/>
-      <c r="G59" s="136"/>
-      <c r="H59" s="136"/>
-      <c r="I59" s="136"/>
-      <c r="J59" s="136"/>
-      <c r="K59" s="136"/>
-      <c r="L59" s="136"/>
-      <c r="M59" s="137"/>
+      <c r="A59" s="149"/>
+      <c r="B59" s="150"/>
+      <c r="C59" s="150"/>
+      <c r="D59" s="150"/>
+      <c r="E59" s="150"/>
+      <c r="F59" s="150"/>
+      <c r="G59" s="150"/>
+      <c r="H59" s="150"/>
+      <c r="I59" s="150"/>
+      <c r="J59" s="150"/>
+      <c r="K59" s="150"/>
+      <c r="L59" s="150"/>
+      <c r="M59" s="151"/>
     </row>
     <row r="60" spans="1:257" s="27" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A60" s="138"/>
-      <c r="B60" s="139"/>
-      <c r="C60" s="139"/>
-      <c r="D60" s="139"/>
-      <c r="E60" s="139"/>
-      <c r="F60" s="139"/>
-      <c r="G60" s="139"/>
-      <c r="H60" s="139"/>
-      <c r="I60" s="139"/>
-      <c r="J60" s="139"/>
-      <c r="K60" s="139"/>
-      <c r="L60" s="139"/>
-      <c r="M60" s="140"/>
+      <c r="A60" s="152"/>
+      <c r="B60" s="153"/>
+      <c r="C60" s="153"/>
+      <c r="D60" s="153"/>
+      <c r="E60" s="153"/>
+      <c r="F60" s="153"/>
+      <c r="G60" s="153"/>
+      <c r="H60" s="153"/>
+      <c r="I60" s="153"/>
+      <c r="J60" s="153"/>
+      <c r="K60" s="153"/>
+      <c r="L60" s="153"/>
+      <c r="M60" s="154"/>
     </row>
     <row r="61" spans="1:257" s="27" customFormat="1">
       <c r="A61" s="9"/>
@@ -4779,7 +4804,7 @@
       <c r="L86" s="10"/>
       <c r="M86" s="11"/>
     </row>
-    <row r="87" spans="1:13" s="27" customFormat="1" ht="28.5">
+    <row r="87" spans="1:13" s="27" customFormat="1" ht="42.75">
       <c r="A87" s="23">
         <v>23</v>
       </c>
@@ -4791,12 +4816,12 @@
         <v>52</v>
       </c>
       <c r="E87" s="22"/>
-      <c r="F87" s="157" t="s">
+      <c r="F87" s="133" t="s">
         <v>55</v>
       </c>
-      <c r="G87" s="157"/>
-      <c r="H87" s="157"/>
-      <c r="I87" s="157"/>
+      <c r="G87" s="133"/>
+      <c r="H87" s="133"/>
+      <c r="I87" s="133"/>
       <c r="J87" s="1"/>
       <c r="K87" s="3"/>
       <c r="L87" s="10"/>
@@ -5087,11 +5112,57 @@
   </sheetData>
   <autoFilter ref="A23:IW24" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <mergeCells count="72">
-    <mergeCell ref="B48:B49"/>
-    <mergeCell ref="E48:E49"/>
-    <mergeCell ref="C48:C49"/>
-    <mergeCell ref="F35:F36"/>
-    <mergeCell ref="G35:G36"/>
+    <mergeCell ref="L35:L36"/>
+    <mergeCell ref="M35:M36"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="H38:I38"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A57:M60"/>
+    <mergeCell ref="C6:L6"/>
+    <mergeCell ref="L10:L11"/>
+    <mergeCell ref="C22:C23"/>
+    <mergeCell ref="D22:D23"/>
+    <mergeCell ref="L48:L49"/>
+    <mergeCell ref="H48:I49"/>
+    <mergeCell ref="L22:L23"/>
+    <mergeCell ref="D48:D49"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="I20:J20"/>
+    <mergeCell ref="B46:M46"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="E22:E23"/>
+    <mergeCell ref="E35:E36"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="B35:B36"/>
+    <mergeCell ref="C35:C36"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="J52:K52"/>
+    <mergeCell ref="J54:K54"/>
+    <mergeCell ref="D35:D36"/>
+    <mergeCell ref="J35:K36"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="H54:I54"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="J48:K49"/>
+    <mergeCell ref="J50:K50"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="H42:I42"/>
     <mergeCell ref="F87:I87"/>
     <mergeCell ref="H55:I55"/>
     <mergeCell ref="H51:I51"/>
@@ -5108,57 +5179,11 @@
     <mergeCell ref="H39:I39"/>
     <mergeCell ref="J55:K55"/>
     <mergeCell ref="J51:K51"/>
-    <mergeCell ref="J52:K52"/>
-    <mergeCell ref="J54:K54"/>
-    <mergeCell ref="D35:D36"/>
-    <mergeCell ref="J35:K36"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="J41:K41"/>
-    <mergeCell ref="J42:K42"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="H54:I54"/>
-    <mergeCell ref="H50:I50"/>
-    <mergeCell ref="J48:K49"/>
-    <mergeCell ref="J50:K50"/>
-    <mergeCell ref="H52:I52"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="E22:E23"/>
-    <mergeCell ref="E35:E36"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="B35:B36"/>
-    <mergeCell ref="C35:C36"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="J39:K39"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="A57:M60"/>
-    <mergeCell ref="C6:L6"/>
-    <mergeCell ref="L10:L11"/>
-    <mergeCell ref="C22:C23"/>
-    <mergeCell ref="D22:D23"/>
-    <mergeCell ref="L48:L49"/>
-    <mergeCell ref="H48:I49"/>
-    <mergeCell ref="L22:L23"/>
-    <mergeCell ref="D48:D49"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="B46:M46"/>
-    <mergeCell ref="L35:L36"/>
-    <mergeCell ref="M35:M36"/>
-    <mergeCell ref="H37:I37"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="H38:I38"/>
-    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="B48:B49"/>
+    <mergeCell ref="E48:E49"/>
+    <mergeCell ref="C48:C49"/>
+    <mergeCell ref="F35:F36"/>
+    <mergeCell ref="G35:G36"/>
   </mergeCells>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
@@ -5548,38 +5573,38 @@
       <c r="M1" s="3"/>
     </row>
     <row r="2" spans="1:13" s="27" customFormat="1" ht="18">
-      <c r="A2" s="130" t="s">
+      <c r="A2" s="144" t="s">
         <v>74</v>
       </c>
-      <c r="B2" s="130"/>
-      <c r="C2" s="130"/>
-      <c r="D2" s="130"/>
-      <c r="E2" s="130"/>
-      <c r="F2" s="130"/>
-      <c r="G2" s="130"/>
-      <c r="H2" s="130"/>
-      <c r="I2" s="130"/>
-      <c r="J2" s="130"/>
-      <c r="K2" s="130"/>
-      <c r="L2" s="130"/>
-      <c r="M2" s="130"/>
+      <c r="B2" s="144"/>
+      <c r="C2" s="144"/>
+      <c r="D2" s="144"/>
+      <c r="E2" s="144"/>
+      <c r="F2" s="144"/>
+      <c r="G2" s="144"/>
+      <c r="H2" s="144"/>
+      <c r="I2" s="144"/>
+      <c r="J2" s="144"/>
+      <c r="K2" s="144"/>
+      <c r="L2" s="144"/>
+      <c r="M2" s="144"/>
     </row>
     <row r="3" spans="1:13" s="27" customFormat="1" ht="15.75" customHeight="1">
-      <c r="A3" s="130" t="s">
+      <c r="A3" s="144" t="s">
         <v>143</v>
       </c>
-      <c r="B3" s="130"/>
-      <c r="C3" s="130"/>
-      <c r="D3" s="130"/>
-      <c r="E3" s="130"/>
-      <c r="F3" s="130"/>
-      <c r="G3" s="130"/>
-      <c r="H3" s="130"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="130"/>
-      <c r="K3" s="130"/>
-      <c r="L3" s="130"/>
-      <c r="M3" s="130"/>
+      <c r="B3" s="144"/>
+      <c r="C3" s="144"/>
+      <c r="D3" s="144"/>
+      <c r="E3" s="144"/>
+      <c r="F3" s="144"/>
+      <c r="G3" s="144"/>
+      <c r="H3" s="144"/>
+      <c r="I3" s="144"/>
+      <c r="J3" s="144"/>
+      <c r="K3" s="144"/>
+      <c r="L3" s="144"/>
+      <c r="M3" s="144"/>
     </row>
     <row r="4" spans="1:13" s="27" customFormat="1" ht="15" customHeight="1">
       <c r="A4" s="1"/>
@@ -5616,16 +5641,16 @@
       <c r="B6" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="141"/>
-      <c r="D6" s="141"/>
-      <c r="E6" s="141"/>
-      <c r="F6" s="141"/>
-      <c r="G6" s="141"/>
-      <c r="H6" s="141"/>
-      <c r="I6" s="141"/>
-      <c r="J6" s="141"/>
-      <c r="K6" s="141"/>
-      <c r="L6" s="141"/>
+      <c r="C6" s="155"/>
+      <c r="D6" s="155"/>
+      <c r="E6" s="155"/>
+      <c r="F6" s="155"/>
+      <c r="G6" s="155"/>
+      <c r="H6" s="155"/>
+      <c r="I6" s="155"/>
+      <c r="J6" s="155"/>
+      <c r="K6" s="155"/>
+      <c r="L6" s="155"/>
       <c r="M6" s="3"/>
     </row>
     <row r="7" spans="1:13" s="27" customFormat="1" ht="15.75">
@@ -5656,10 +5681,10 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
-      <c r="I8" s="150" t="s">
+      <c r="I8" s="156" t="s">
         <v>36</v>
       </c>
-      <c r="J8" s="150"/>
+      <c r="J8" s="156"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="3"/>
@@ -5681,50 +5706,50 @@
     </row>
     <row r="10" spans="1:13" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A10" s="35"/>
-      <c r="B10" s="142" t="s">
+      <c r="B10" s="131" t="s">
         <v>144</v>
       </c>
-      <c r="C10" s="142" t="s">
+      <c r="C10" s="131" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="142" t="s">
+      <c r="D10" s="131" t="s">
         <v>25</v>
       </c>
-      <c r="E10" s="127" t="s">
+      <c r="E10" s="129" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="142" t="s">
+      <c r="F10" s="131" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="142" t="s">
+      <c r="G10" s="131" t="s">
         <v>24</v>
       </c>
       <c r="H10" s="1"/>
-      <c r="I10" s="152" t="s">
+      <c r="I10" s="136" t="s">
         <v>31</v>
       </c>
-      <c r="J10" s="142" t="s">
+      <c r="J10" s="131" t="s">
         <v>32</v>
       </c>
       <c r="K10" s="120"/>
-      <c r="L10" s="142" t="s">
+      <c r="L10" s="131" t="s">
         <v>37</v>
       </c>
       <c r="M10" s="3"/>
     </row>
     <row r="11" spans="1:13" s="27" customFormat="1" ht="28.35" customHeight="1">
       <c r="A11" s="35"/>
-      <c r="B11" s="143"/>
-      <c r="C11" s="143"/>
-      <c r="D11" s="143"/>
-      <c r="E11" s="155"/>
-      <c r="F11" s="143"/>
-      <c r="G11" s="143"/>
+      <c r="B11" s="132"/>
+      <c r="C11" s="132"/>
+      <c r="D11" s="132"/>
+      <c r="E11" s="130"/>
+      <c r="F11" s="132"/>
+      <c r="G11" s="132"/>
       <c r="H11" s="1"/>
-      <c r="I11" s="153"/>
-      <c r="J11" s="143"/>
+      <c r="I11" s="137"/>
+      <c r="J11" s="132"/>
       <c r="K11" s="120"/>
-      <c r="L11" s="143"/>
+      <c r="L11" s="132"/>
       <c r="M11" s="3"/>
     </row>
     <row r="12" spans="1:13" s="27" customFormat="1" ht="15.95" customHeight="1">
@@ -6010,10 +6035,10 @@
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
-      <c r="I30" s="150" t="s">
+      <c r="I30" s="156" t="s">
         <v>36</v>
       </c>
-      <c r="J30" s="150"/>
+      <c r="J30" s="156"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="3"/>
@@ -6035,53 +6060,53 @@
     </row>
     <row r="32" spans="1:13" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A32" s="35"/>
-      <c r="B32" s="142" t="s">
+      <c r="B32" s="131" t="s">
         <v>144</v>
       </c>
-      <c r="C32" s="142" t="s">
+      <c r="C32" s="131" t="s">
         <v>26</v>
       </c>
-      <c r="D32" s="142" t="s">
+      <c r="D32" s="131" t="s">
         <v>25</v>
       </c>
-      <c r="E32" s="127" t="s">
+      <c r="E32" s="129" t="s">
         <v>114</v>
       </c>
-      <c r="F32" s="142" t="s">
+      <c r="F32" s="131" t="s">
         <v>27</v>
       </c>
-      <c r="G32" s="142" t="s">
+      <c r="G32" s="131" t="s">
         <v>24</v>
       </c>
       <c r="H32" s="1"/>
-      <c r="I32" s="152" t="s">
+      <c r="I32" s="136" t="s">
         <v>31</v>
       </c>
-      <c r="J32" s="142" t="s">
+      <c r="J32" s="131" t="s">
         <v>32</v>
       </c>
       <c r="K32" s="120"/>
-      <c r="L32" s="142" t="s">
+      <c r="L32" s="131" t="s">
         <v>38</v>
       </c>
-      <c r="M32" s="142" t="s">
+      <c r="M32" s="131" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="33" spans="1:13" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A33" s="35"/>
-      <c r="B33" s="143"/>
-      <c r="C33" s="143"/>
-      <c r="D33" s="143"/>
-      <c r="E33" s="155"/>
-      <c r="F33" s="143"/>
-      <c r="G33" s="143"/>
+      <c r="B33" s="132"/>
+      <c r="C33" s="132"/>
+      <c r="D33" s="132"/>
+      <c r="E33" s="130"/>
+      <c r="F33" s="132"/>
+      <c r="G33" s="132"/>
       <c r="H33" s="1"/>
-      <c r="I33" s="153"/>
-      <c r="J33" s="143"/>
+      <c r="I33" s="137"/>
+      <c r="J33" s="132"/>
       <c r="K33" s="120"/>
-      <c r="L33" s="143"/>
-      <c r="M33" s="143"/>
+      <c r="L33" s="132"/>
+      <c r="M33" s="132"/>
     </row>
     <row r="34" spans="1:13" s="27" customFormat="1" ht="15.95" customHeight="1">
       <c r="A34" s="35"/>
@@ -6726,10 +6751,10 @@
       <c r="A76" s="37" t="s">
         <v>70</v>
       </c>
-      <c r="B76" s="131" t="s">
+      <c r="B76" s="145" t="s">
         <v>66</v>
       </c>
-      <c r="C76" s="131"/>
+      <c r="C76" s="145"/>
       <c r="D76" s="1"/>
       <c r="E76" s="1"/>
       <c r="F76" s="29"/>
@@ -6758,53 +6783,53 @@
     </row>
     <row r="78" spans="1:13" s="27" customFormat="1" ht="15.75">
       <c r="A78" s="35"/>
-      <c r="B78" s="142" t="s">
+      <c r="B78" s="131" t="s">
         <v>144</v>
       </c>
-      <c r="C78" s="142" t="s">
+      <c r="C78" s="131" t="s">
         <v>26</v>
       </c>
-      <c r="D78" s="142" t="s">
+      <c r="D78" s="131" t="s">
         <v>113</v>
       </c>
-      <c r="E78" s="127" t="s">
+      <c r="E78" s="129" t="s">
         <v>114</v>
       </c>
-      <c r="F78" s="142" t="s">
+      <c r="F78" s="131" t="s">
         <v>27</v>
       </c>
-      <c r="G78" s="142" t="s">
+      <c r="G78" s="131" t="s">
         <v>24</v>
       </c>
-      <c r="H78" s="144" t="s">
+      <c r="H78" s="138" t="s">
         <v>138</v>
       </c>
-      <c r="I78" s="145"/>
-      <c r="J78" s="144" t="s">
+      <c r="I78" s="139"/>
+      <c r="J78" s="138" t="s">
         <v>139</v>
       </c>
-      <c r="K78" s="145"/>
-      <c r="L78" s="127" t="s">
+      <c r="K78" s="139"/>
+      <c r="L78" s="129" t="s">
         <v>140</v>
       </c>
-      <c r="M78" s="127" t="s">
+      <c r="M78" s="129" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="79" spans="1:13" s="27" customFormat="1" ht="15.75">
       <c r="A79" s="35"/>
-      <c r="B79" s="143"/>
-      <c r="C79" s="143"/>
-      <c r="D79" s="143"/>
-      <c r="E79" s="155"/>
-      <c r="F79" s="143"/>
-      <c r="G79" s="143"/>
-      <c r="H79" s="146"/>
-      <c r="I79" s="147"/>
-      <c r="J79" s="146"/>
-      <c r="K79" s="147"/>
-      <c r="L79" s="128"/>
-      <c r="M79" s="128"/>
+      <c r="B79" s="132"/>
+      <c r="C79" s="132"/>
+      <c r="D79" s="132"/>
+      <c r="E79" s="130"/>
+      <c r="F79" s="132"/>
+      <c r="G79" s="132"/>
+      <c r="H79" s="140"/>
+      <c r="I79" s="141"/>
+      <c r="J79" s="140"/>
+      <c r="K79" s="141"/>
+      <c r="L79" s="135"/>
+      <c r="M79" s="135"/>
     </row>
     <row r="80" spans="1:13" s="27" customFormat="1" ht="15.75">
       <c r="A80" s="35"/>
@@ -6814,10 +6839,10 @@
       <c r="E80" s="6"/>
       <c r="F80" s="6"/>
       <c r="G80" s="6"/>
-      <c r="H80" s="129"/>
-      <c r="I80" s="129"/>
-      <c r="J80" s="129"/>
-      <c r="K80" s="129"/>
+      <c r="H80" s="134"/>
+      <c r="I80" s="134"/>
+      <c r="J80" s="134"/>
+      <c r="K80" s="134"/>
       <c r="L80" s="7"/>
       <c r="M80" s="7"/>
     </row>
@@ -6829,10 +6854,10 @@
       <c r="E81" s="6"/>
       <c r="F81" s="6"/>
       <c r="G81" s="6"/>
-      <c r="H81" s="129"/>
-      <c r="I81" s="129"/>
-      <c r="J81" s="129"/>
-      <c r="K81" s="129"/>
+      <c r="H81" s="134"/>
+      <c r="I81" s="134"/>
+      <c r="J81" s="134"/>
+      <c r="K81" s="134"/>
       <c r="L81" s="7"/>
       <c r="M81" s="7"/>
     </row>
@@ -6844,10 +6869,10 @@
       <c r="E82" s="6"/>
       <c r="F82" s="6"/>
       <c r="G82" s="6"/>
-      <c r="H82" s="129"/>
-      <c r="I82" s="129"/>
-      <c r="J82" s="129"/>
-      <c r="K82" s="129"/>
+      <c r="H82" s="134"/>
+      <c r="I82" s="134"/>
+      <c r="J82" s="134"/>
+      <c r="K82" s="134"/>
       <c r="L82" s="7"/>
       <c r="M82" s="7"/>
     </row>
@@ -6859,10 +6884,10 @@
       <c r="E83" s="6"/>
       <c r="F83" s="6"/>
       <c r="G83" s="36"/>
-      <c r="H83" s="129"/>
-      <c r="I83" s="129"/>
-      <c r="J83" s="154"/>
-      <c r="K83" s="154"/>
+      <c r="H83" s="134"/>
+      <c r="I83" s="134"/>
+      <c r="J83" s="143"/>
+      <c r="K83" s="143"/>
       <c r="L83" s="7"/>
       <c r="M83" s="7"/>
     </row>
@@ -6874,10 +6899,10 @@
       <c r="E84" s="6"/>
       <c r="F84" s="6"/>
       <c r="G84" s="6"/>
-      <c r="H84" s="129"/>
-      <c r="I84" s="129"/>
-      <c r="J84" s="129"/>
-      <c r="K84" s="129"/>
+      <c r="H84" s="134"/>
+      <c r="I84" s="134"/>
+      <c r="J84" s="134"/>
+      <c r="K84" s="134"/>
       <c r="L84" s="7"/>
       <c r="M84" s="7"/>
     </row>
@@ -6889,10 +6914,10 @@
       <c r="E85" s="6"/>
       <c r="F85" s="6"/>
       <c r="G85" s="6"/>
-      <c r="H85" s="129"/>
-      <c r="I85" s="129"/>
-      <c r="J85" s="129"/>
-      <c r="K85" s="129"/>
+      <c r="H85" s="134"/>
+      <c r="I85" s="134"/>
+      <c r="J85" s="134"/>
+      <c r="K85" s="134"/>
       <c r="L85" s="7"/>
       <c r="M85" s="7"/>
     </row>
@@ -6947,20 +6972,20 @@
     </row>
     <row r="89" spans="1:13" s="27" customFormat="1" ht="39.75" customHeight="1">
       <c r="A89" s="1"/>
-      <c r="B89" s="151" t="s">
+      <c r="B89" s="157" t="s">
         <v>142</v>
       </c>
-      <c r="C89" s="151"/>
-      <c r="D89" s="151"/>
-      <c r="E89" s="151"/>
-      <c r="F89" s="151"/>
-      <c r="G89" s="151"/>
-      <c r="H89" s="151"/>
-      <c r="I89" s="151"/>
-      <c r="J89" s="151"/>
-      <c r="K89" s="151"/>
-      <c r="L89" s="151"/>
-      <c r="M89" s="151"/>
+      <c r="C89" s="157"/>
+      <c r="D89" s="157"/>
+      <c r="E89" s="157"/>
+      <c r="F89" s="157"/>
+      <c r="G89" s="157"/>
+      <c r="H89" s="157"/>
+      <c r="I89" s="157"/>
+      <c r="J89" s="157"/>
+      <c r="K89" s="157"/>
+      <c r="L89" s="157"/>
+      <c r="M89" s="157"/>
     </row>
     <row r="90" spans="1:13" s="27" customFormat="1" ht="16.5" customHeight="1">
       <c r="A90" s="1"/>
@@ -6979,53 +7004,53 @@
     </row>
     <row r="91" spans="1:13" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A91" s="1"/>
-      <c r="B91" s="142" t="s">
+      <c r="B91" s="131" t="s">
         <v>144</v>
       </c>
-      <c r="C91" s="148" t="s">
+      <c r="C91" s="127" t="s">
         <v>26</v>
       </c>
-      <c r="D91" s="148" t="s">
+      <c r="D91" s="127" t="s">
         <v>25</v>
       </c>
-      <c r="E91" s="127" t="s">
+      <c r="E91" s="129" t="s">
         <v>114</v>
       </c>
-      <c r="F91" s="148" t="s">
+      <c r="F91" s="127" t="s">
         <v>27</v>
       </c>
-      <c r="G91" s="148" t="s">
+      <c r="G91" s="127" t="s">
         <v>24</v>
       </c>
-      <c r="H91" s="144" t="s">
+      <c r="H91" s="138" t="s">
         <v>138</v>
       </c>
-      <c r="I91" s="145"/>
-      <c r="J91" s="144" t="s">
+      <c r="I91" s="139"/>
+      <c r="J91" s="138" t="s">
         <v>139</v>
       </c>
-      <c r="K91" s="145"/>
-      <c r="L91" s="127" t="s">
+      <c r="K91" s="139"/>
+      <c r="L91" s="129" t="s">
         <v>140</v>
       </c>
-      <c r="M91" s="127" t="s">
+      <c r="M91" s="129" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="92" spans="1:13" s="27" customFormat="1" ht="18" customHeight="1">
       <c r="A92" s="1"/>
-      <c r="B92" s="143"/>
-      <c r="C92" s="149"/>
-      <c r="D92" s="149"/>
-      <c r="E92" s="155"/>
-      <c r="F92" s="149"/>
-      <c r="G92" s="149"/>
-      <c r="H92" s="146"/>
-      <c r="I92" s="147"/>
-      <c r="J92" s="146"/>
-      <c r="K92" s="147"/>
-      <c r="L92" s="128"/>
-      <c r="M92" s="128"/>
+      <c r="B92" s="132"/>
+      <c r="C92" s="128"/>
+      <c r="D92" s="128"/>
+      <c r="E92" s="130"/>
+      <c r="F92" s="128"/>
+      <c r="G92" s="128"/>
+      <c r="H92" s="140"/>
+      <c r="I92" s="141"/>
+      <c r="J92" s="140"/>
+      <c r="K92" s="141"/>
+      <c r="L92" s="135"/>
+      <c r="M92" s="135"/>
     </row>
     <row r="93" spans="1:13" s="108" customFormat="1" ht="15.95" customHeight="1">
       <c r="B93" s="70"/>
@@ -7033,10 +7058,10 @@
       <c r="D93" s="109"/>
       <c r="F93" s="114"/>
       <c r="G93" s="110"/>
-      <c r="H93" s="156"/>
-      <c r="I93" s="156"/>
-      <c r="J93" s="156"/>
-      <c r="K93" s="156"/>
+      <c r="H93" s="142"/>
+      <c r="I93" s="142"/>
+      <c r="J93" s="142"/>
+      <c r="K93" s="142"/>
       <c r="L93" s="109"/>
       <c r="M93" s="109"/>
     </row>
@@ -7048,10 +7073,10 @@
       <c r="E94" s="6"/>
       <c r="F94" s="6"/>
       <c r="G94" s="6"/>
-      <c r="H94" s="129"/>
-      <c r="I94" s="129"/>
-      <c r="J94" s="129"/>
-      <c r="K94" s="129"/>
+      <c r="H94" s="134"/>
+      <c r="I94" s="134"/>
+      <c r="J94" s="134"/>
+      <c r="K94" s="134"/>
       <c r="L94" s="7"/>
       <c r="M94" s="7"/>
     </row>
@@ -7063,10 +7088,10 @@
       <c r="E95" s="6"/>
       <c r="F95" s="6"/>
       <c r="G95" s="6"/>
-      <c r="H95" s="129"/>
-      <c r="I95" s="129"/>
-      <c r="J95" s="129"/>
-      <c r="K95" s="129"/>
+      <c r="H95" s="134"/>
+      <c r="I95" s="134"/>
+      <c r="J95" s="134"/>
+      <c r="K95" s="134"/>
       <c r="L95" s="7"/>
       <c r="M95" s="7"/>
     </row>
@@ -7078,10 +7103,10 @@
       <c r="E96" s="6"/>
       <c r="F96" s="6"/>
       <c r="G96" s="6"/>
-      <c r="H96" s="129"/>
-      <c r="I96" s="129"/>
-      <c r="J96" s="129"/>
-      <c r="K96" s="129"/>
+      <c r="H96" s="134"/>
+      <c r="I96" s="134"/>
+      <c r="J96" s="134"/>
+      <c r="K96" s="134"/>
       <c r="L96" s="7"/>
       <c r="M96" s="7"/>
     </row>
@@ -7093,10 +7118,10 @@
       <c r="E97" s="6"/>
       <c r="F97" s="6"/>
       <c r="G97" s="6"/>
-      <c r="H97" s="129"/>
-      <c r="I97" s="129"/>
-      <c r="J97" s="129"/>
-      <c r="K97" s="129"/>
+      <c r="H97" s="134"/>
+      <c r="I97" s="134"/>
+      <c r="J97" s="134"/>
+      <c r="K97" s="134"/>
       <c r="L97" s="7"/>
       <c r="M97" s="7"/>
     </row>
@@ -7108,10 +7133,10 @@
       <c r="E98" s="6"/>
       <c r="F98" s="6"/>
       <c r="G98" s="6"/>
-      <c r="H98" s="129"/>
-      <c r="I98" s="129"/>
-      <c r="J98" s="129"/>
-      <c r="K98" s="129"/>
+      <c r="H98" s="134"/>
+      <c r="I98" s="134"/>
+      <c r="J98" s="134"/>
+      <c r="K98" s="134"/>
       <c r="L98" s="7"/>
       <c r="M98" s="7"/>
     </row>
@@ -7131,21 +7156,21 @@
       <c r="M99" s="3"/>
     </row>
     <row r="100" spans="1:257" s="1" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A100" s="132" t="s">
+      <c r="A100" s="146" t="s">
         <v>21</v>
       </c>
-      <c r="B100" s="133"/>
-      <c r="C100" s="133"/>
-      <c r="D100" s="133"/>
-      <c r="E100" s="133"/>
-      <c r="F100" s="133"/>
-      <c r="G100" s="133"/>
-      <c r="H100" s="133"/>
-      <c r="I100" s="133"/>
-      <c r="J100" s="133"/>
-      <c r="K100" s="133"/>
-      <c r="L100" s="133"/>
-      <c r="M100" s="134"/>
+      <c r="B100" s="147"/>
+      <c r="C100" s="147"/>
+      <c r="D100" s="147"/>
+      <c r="E100" s="147"/>
+      <c r="F100" s="147"/>
+      <c r="G100" s="147"/>
+      <c r="H100" s="147"/>
+      <c r="I100" s="147"/>
+      <c r="J100" s="147"/>
+      <c r="K100" s="147"/>
+      <c r="L100" s="147"/>
+      <c r="M100" s="148"/>
       <c r="N100" s="27"/>
       <c r="O100" s="27"/>
       <c r="P100" s="27"/>
@@ -7392,49 +7417,49 @@
       <c r="IW100" s="27"/>
     </row>
     <row r="101" spans="1:257" s="27" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A101" s="135"/>
-      <c r="B101" s="136"/>
-      <c r="C101" s="136"/>
-      <c r="D101" s="136"/>
-      <c r="E101" s="136"/>
-      <c r="F101" s="136"/>
-      <c r="G101" s="136"/>
-      <c r="H101" s="136"/>
-      <c r="I101" s="136"/>
-      <c r="J101" s="136"/>
-      <c r="K101" s="136"/>
-      <c r="L101" s="136"/>
-      <c r="M101" s="137"/>
+      <c r="A101" s="149"/>
+      <c r="B101" s="150"/>
+      <c r="C101" s="150"/>
+      <c r="D101" s="150"/>
+      <c r="E101" s="150"/>
+      <c r="F101" s="150"/>
+      <c r="G101" s="150"/>
+      <c r="H101" s="150"/>
+      <c r="I101" s="150"/>
+      <c r="J101" s="150"/>
+      <c r="K101" s="150"/>
+      <c r="L101" s="150"/>
+      <c r="M101" s="151"/>
     </row>
     <row r="102" spans="1:257" s="27" customFormat="1" ht="12.75" customHeight="1">
-      <c r="A102" s="135"/>
-      <c r="B102" s="136"/>
-      <c r="C102" s="136"/>
-      <c r="D102" s="136"/>
-      <c r="E102" s="136"/>
-      <c r="F102" s="136"/>
-      <c r="G102" s="136"/>
-      <c r="H102" s="136"/>
-      <c r="I102" s="136"/>
-      <c r="J102" s="136"/>
-      <c r="K102" s="136"/>
-      <c r="L102" s="136"/>
-      <c r="M102" s="137"/>
+      <c r="A102" s="149"/>
+      <c r="B102" s="150"/>
+      <c r="C102" s="150"/>
+      <c r="D102" s="150"/>
+      <c r="E102" s="150"/>
+      <c r="F102" s="150"/>
+      <c r="G102" s="150"/>
+      <c r="H102" s="150"/>
+      <c r="I102" s="150"/>
+      <c r="J102" s="150"/>
+      <c r="K102" s="150"/>
+      <c r="L102" s="150"/>
+      <c r="M102" s="151"/>
     </row>
     <row r="103" spans="1:257" s="27" customFormat="1" ht="12.75" customHeight="1" thickBot="1">
-      <c r="A103" s="138"/>
-      <c r="B103" s="139"/>
-      <c r="C103" s="139"/>
-      <c r="D103" s="139"/>
-      <c r="E103" s="139"/>
-      <c r="F103" s="139"/>
-      <c r="G103" s="139"/>
-      <c r="H103" s="139"/>
-      <c r="I103" s="139"/>
-      <c r="J103" s="139"/>
-      <c r="K103" s="139"/>
-      <c r="L103" s="139"/>
-      <c r="M103" s="140"/>
+      <c r="A103" s="152"/>
+      <c r="B103" s="153"/>
+      <c r="C103" s="153"/>
+      <c r="D103" s="153"/>
+      <c r="E103" s="153"/>
+      <c r="F103" s="153"/>
+      <c r="G103" s="153"/>
+      <c r="H103" s="153"/>
+      <c r="I103" s="153"/>
+      <c r="J103" s="153"/>
+      <c r="K103" s="153"/>
+      <c r="L103" s="153"/>
+      <c r="M103" s="154"/>
     </row>
     <row r="104" spans="1:257" s="27" customFormat="1">
       <c r="A104" s="9"/>
@@ -8022,12 +8047,12 @@
         <v>52</v>
       </c>
       <c r="E130" s="22"/>
-      <c r="F130" s="157" t="s">
+      <c r="F130" s="133" t="s">
         <v>55</v>
       </c>
-      <c r="G130" s="157"/>
-      <c r="H130" s="157"/>
-      <c r="I130" s="157"/>
+      <c r="G130" s="133"/>
+      <c r="H130" s="133"/>
+      <c r="I130" s="133"/>
       <c r="J130" s="1"/>
       <c r="K130" s="3"/>
       <c r="L130" s="10"/>
@@ -8322,6 +8347,62 @@
     </sortState>
   </autoFilter>
   <mergeCells count="72">
+    <mergeCell ref="A2:M2"/>
+    <mergeCell ref="A3:M3"/>
+    <mergeCell ref="C6:L6"/>
+    <mergeCell ref="I8:J8"/>
+    <mergeCell ref="B10:B11"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="F10:F11"/>
+    <mergeCell ref="G10:G11"/>
+    <mergeCell ref="I10:I11"/>
+    <mergeCell ref="J10:J11"/>
+    <mergeCell ref="L10:L11"/>
+    <mergeCell ref="I30:J30"/>
+    <mergeCell ref="B32:B33"/>
+    <mergeCell ref="C32:C33"/>
+    <mergeCell ref="D32:D33"/>
+    <mergeCell ref="E32:E33"/>
+    <mergeCell ref="F32:F33"/>
+    <mergeCell ref="G32:G33"/>
+    <mergeCell ref="M32:M33"/>
+    <mergeCell ref="B76:C76"/>
+    <mergeCell ref="B78:B79"/>
+    <mergeCell ref="C78:C79"/>
+    <mergeCell ref="D78:D79"/>
+    <mergeCell ref="E78:E79"/>
+    <mergeCell ref="F78:F79"/>
+    <mergeCell ref="G78:G79"/>
+    <mergeCell ref="M78:M79"/>
+    <mergeCell ref="H80:I80"/>
+    <mergeCell ref="J80:K80"/>
+    <mergeCell ref="I32:I33"/>
+    <mergeCell ref="J32:J33"/>
+    <mergeCell ref="L32:L33"/>
+    <mergeCell ref="H78:I79"/>
+    <mergeCell ref="J78:K79"/>
+    <mergeCell ref="L78:L79"/>
+    <mergeCell ref="H91:I92"/>
+    <mergeCell ref="J91:K92"/>
+    <mergeCell ref="L91:L92"/>
+    <mergeCell ref="H81:I81"/>
+    <mergeCell ref="J81:K81"/>
+    <mergeCell ref="H82:I82"/>
+    <mergeCell ref="J82:K82"/>
+    <mergeCell ref="H83:I83"/>
+    <mergeCell ref="J83:K83"/>
+    <mergeCell ref="C91:C92"/>
+    <mergeCell ref="D91:D92"/>
+    <mergeCell ref="E91:E92"/>
+    <mergeCell ref="F91:F92"/>
+    <mergeCell ref="G91:G92"/>
+    <mergeCell ref="H84:I84"/>
+    <mergeCell ref="J84:K84"/>
+    <mergeCell ref="H85:I85"/>
+    <mergeCell ref="J85:K85"/>
+    <mergeCell ref="B89:M89"/>
     <mergeCell ref="M91:M92"/>
     <mergeCell ref="F130:I130"/>
     <mergeCell ref="H94:I94"/>
@@ -8337,63 +8418,7 @@
     <mergeCell ref="A100:M103"/>
     <mergeCell ref="H93:I93"/>
     <mergeCell ref="J93:K93"/>
-    <mergeCell ref="H84:I84"/>
-    <mergeCell ref="J84:K84"/>
-    <mergeCell ref="H85:I85"/>
-    <mergeCell ref="J85:K85"/>
-    <mergeCell ref="B89:M89"/>
     <mergeCell ref="B91:B92"/>
-    <mergeCell ref="C91:C92"/>
-    <mergeCell ref="D91:D92"/>
-    <mergeCell ref="E91:E92"/>
-    <mergeCell ref="F91:F92"/>
-    <mergeCell ref="G91:G92"/>
-    <mergeCell ref="H91:I92"/>
-    <mergeCell ref="J91:K92"/>
-    <mergeCell ref="L91:L92"/>
-    <mergeCell ref="H81:I81"/>
-    <mergeCell ref="J81:K81"/>
-    <mergeCell ref="H82:I82"/>
-    <mergeCell ref="J82:K82"/>
-    <mergeCell ref="H83:I83"/>
-    <mergeCell ref="J83:K83"/>
-    <mergeCell ref="H80:I80"/>
-    <mergeCell ref="J80:K80"/>
-    <mergeCell ref="I32:I33"/>
-    <mergeCell ref="J32:J33"/>
-    <mergeCell ref="L32:L33"/>
-    <mergeCell ref="H78:I79"/>
-    <mergeCell ref="J78:K79"/>
-    <mergeCell ref="L78:L79"/>
-    <mergeCell ref="M32:M33"/>
-    <mergeCell ref="B76:C76"/>
-    <mergeCell ref="B78:B79"/>
-    <mergeCell ref="C78:C79"/>
-    <mergeCell ref="D78:D79"/>
-    <mergeCell ref="E78:E79"/>
-    <mergeCell ref="F78:F79"/>
-    <mergeCell ref="G78:G79"/>
-    <mergeCell ref="M78:M79"/>
-    <mergeCell ref="I30:J30"/>
-    <mergeCell ref="B32:B33"/>
-    <mergeCell ref="C32:C33"/>
-    <mergeCell ref="D32:D33"/>
-    <mergeCell ref="E32:E33"/>
-    <mergeCell ref="F32:F33"/>
-    <mergeCell ref="G32:G33"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A3:M3"/>
-    <mergeCell ref="C6:L6"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="B10:B11"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="F10:F11"/>
-    <mergeCell ref="G10:G11"/>
-    <mergeCell ref="I10:I11"/>
-    <mergeCell ref="J10:J11"/>
-    <mergeCell ref="L10:L11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup scale="41" orientation="landscape" r:id="rId1"/>

</xml_diff>